<commit_message>
refactor naming to add NamingSystems
</commit_message>
<xml_diff>
--- a/StructureDefinition-ng-aefi-report-bundle.xlsx
+++ b/StructureDefinition-ng-aefi-report-bundle.xlsx
@@ -51,7 +51,7 @@
     <t>Title</t>
   </si>
   <si>
-    <t>4-NG AEFI Report Bundle</t>
+    <t>Bundle NG AEFI Report</t>
   </si>
   <si>
     <t>Status</t>
@@ -66,7 +66,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-12T13:22:49+01:00</t>
+    <t>2026-08-17T07:55:48+01:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>